<commit_message>
refactor: update feature traceability matrix, data definitions, and reporting scripts for SolarKits v2.0
</commit_message>
<xml_diff>
--- a/SolarKits_Feature_Traceability_Matrix.xlsx
+++ b/SolarKits_Feature_Traceability_Matrix.xlsx
@@ -65,6 +65,12 @@
     <font>
       <name val="Arial"/>
       <b val="1"/>
+      <color rgb="00D97706"/>
+      <sz val="8.5"/>
+    </font>
+    <font>
+      <name val="Arial"/>
+      <b val="1"/>
       <color rgb="0064748B"/>
       <sz val="8.5"/>
     </font>
@@ -72,12 +78,6 @@
       <name val="Arial"/>
       <b val="1"/>
       <color rgb="00DC2626"/>
-      <sz val="8.5"/>
-    </font>
-    <font>
-      <name val="Arial"/>
-      <b val="1"/>
-      <color rgb="00D97706"/>
       <sz val="8.5"/>
     </font>
   </fonts>
@@ -190,7 +190,7 @@
     <xf numFmtId="0" fontId="9" fillId="0" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="center" vertical="top"/>
     </xf>
-    <xf numFmtId="0" fontId="9" fillId="3" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+    <xf numFmtId="0" fontId="7" fillId="3" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="center" vertical="top"/>
     </xf>
     <xf numFmtId="0" fontId="3" fillId="4" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
@@ -205,13 +205,13 @@
     <xf numFmtId="0" fontId="5" fillId="4" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment vertical="top" wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="7" fillId="4" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+    <xf numFmtId="0" fontId="8" fillId="4" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="center" vertical="top"/>
     </xf>
     <xf numFmtId="0" fontId="6" fillId="4" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="center" vertical="top"/>
     </xf>
-    <xf numFmtId="0" fontId="9" fillId="4" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+    <xf numFmtId="0" fontId="7" fillId="4" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="center" vertical="top"/>
     </xf>
     <xf numFmtId="0" fontId="3" fillId="0" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
@@ -220,7 +220,7 @@
     <xf numFmtId="0" fontId="4" fillId="0" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="center" vertical="top"/>
     </xf>
-    <xf numFmtId="0" fontId="8" fillId="3" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+    <xf numFmtId="0" fontId="9" fillId="3" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="center" vertical="top"/>
     </xf>
     <xf numFmtId="0" fontId="3" fillId="3" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
@@ -229,7 +229,7 @@
     <xf numFmtId="0" fontId="4" fillId="3" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="center" vertical="top"/>
     </xf>
-    <xf numFmtId="0" fontId="7" fillId="3" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+    <xf numFmtId="0" fontId="8" fillId="3" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="center" vertical="top"/>
     </xf>
     <xf numFmtId="0" fontId="4" fillId="0" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
@@ -649,12 +649,12 @@
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="8" customWidth="1" min="1" max="1"/>
-    <col width="18" customWidth="1" min="2" max="2"/>
-    <col width="25" customWidth="1" min="3" max="3"/>
-    <col width="30" customWidth="1" min="4" max="4"/>
-    <col width="32" customWidth="1" min="5" max="5"/>
+    <col width="22" customWidth="1" min="2" max="2"/>
+    <col width="28" customWidth="1" min="3" max="3"/>
+    <col width="32" customWidth="1" min="4" max="4"/>
+    <col width="34" customWidth="1" min="5" max="5"/>
     <col width="18" customWidth="1" min="6" max="6"/>
-    <col width="50" customWidth="1" min="7" max="7"/>
+    <col width="55" customWidth="1" min="7" max="7"/>
   </cols>
   <sheetData>
     <row r="1" ht="25" customHeight="1">
@@ -862,17 +862,17 @@
       </c>
       <c r="C7" s="6" t="inlineStr">
         <is>
-          <t>BOSKIT Distributor Auth</t>
+          <t>Multi-Role CMS Panel &amp; Scope Authorization</t>
         </is>
       </c>
       <c r="D7" s="7" t="inlineStr">
         <is>
-          <t>boskit-website/LoginPage.jsx</t>
+          <t>internal-admin-portal/src/portals/cms-auth/Login.jsx</t>
         </is>
       </c>
       <c r="E7" s="7" t="inlineStr">
         <is>
-          <t>/api/boskit/v1/auth/*</t>
+          <t>/auth-api/login, cms.auth.handler.js, cms_user_scope.schema.js</t>
         </is>
       </c>
       <c r="F7" s="8" t="inlineStr">
@@ -882,7 +882,7 @@
       </c>
       <c r="G7" s="9" t="inlineStr">
         <is>
-          <t>Multi-tier authentication portal for BOS distributors and local electrical dealers with role-based permission scopes, territory binding, and dealer network association.</t>
+          <t>Enterprise role-based access control granting compartmentalized permissions across Super Admin, Accounts, Warehouse, Operations, Developer, and BDE portals with dynamic panel scope resolution.</t>
         </is>
       </c>
     </row>
@@ -2638,7 +2638,7 @@
       </c>
       <c r="C55" s="6" t="inlineStr">
         <is>
-          <t>Solar BOS Kit (Commented Out)</t>
+          <t>Dynamic Combo Kit BOM Customizer</t>
         </is>
       </c>
       <c r="D55" s="7" t="inlineStr">
@@ -2648,7 +2648,7 @@
       </c>
       <c r="E55" s="7" t="inlineStr">
         <is>
-          <t>/api/india/v1/bos-kits</t>
+          <t>/api/india/v1/combo-kits/customize, product.template.handler.js</t>
         </is>
       </c>
       <c r="F55" s="8" t="inlineStr">
@@ -2658,7 +2658,7 @@
       </c>
       <c r="G55" s="9" t="inlineStr">
         <is>
-          <t>Specialized catalog for Balance of System electrical accessories (DCDB, ACDB, cables, earthing kits) — backend API active; menu item commented in frontend. Full 1,506-line component for ordering electrical BOS distribution components, ACDB/DCDB boxes, MC4 connectors, and solar cabling.</t>
+          <t>Interactive Bill of Materials (BOM) customizer allowing EPC contractors to dynamically configure solar panels, inverters, mounting structures, and electrical balance components with live technical validation.</t>
         </is>
       </c>
     </row>
@@ -2781,22 +2781,22 @@
       </c>
       <c r="B59" s="5" t="inlineStr">
         <is>
-          <t>BOSKIT</t>
+          <t>Kit Activation &amp; Order Settings</t>
         </is>
       </c>
       <c r="C59" s="6" t="inlineStr">
         <is>
-          <t>Distributor Onboarding</t>
+          <t>Warehouse Kit Activation Engine (ADM_WH_KIT_ACT)</t>
         </is>
       </c>
       <c r="D59" s="7" t="inlineStr">
         <is>
-          <t>boskit-website/DistributorOnboardingPage.jsx</t>
+          <t>internal-admin-portal/src/portals/admin/pages/solar-shop/warehouse-kit-activations/WarehouseKitConfig.jsx</t>
         </is>
       </c>
       <c r="E59" s="7" t="inlineStr">
         <is>
-          <t>/api/boskit/v1/distributor/onboarding/*</t>
+          <t>/admin-api/solarshop/warehouse-kit-activations/*, warehouse_kit_activations.handler.js</t>
         </is>
       </c>
       <c r="F59" s="8" t="inlineStr">
@@ -2806,7 +2806,7 @@
       </c>
       <c r="G59" s="9" t="inlineStr">
         <is>
-          <t>Multi-step onboarding wizard for BOS channel distributors featuring GST verification, KYC document uploads, and territory allocation.</t>
+          <t>Stage 1 Warehouse Kit Activation enforcing 3 mandatory prerequisite validation gates (Cluster SKU Benchmark Pricing, Company Profit Margin, GST Rate Configuration) before allowing any kit to become active in a warehouse.</t>
         </is>
       </c>
     </row>
@@ -2818,22 +2818,22 @@
       </c>
       <c r="B60" s="11" t="inlineStr">
         <is>
-          <t>BOSKIT</t>
+          <t>Kit Activation &amp; Order Settings</t>
         </is>
       </c>
       <c r="C60" s="12" t="inlineStr">
         <is>
-          <t>Distributor Plans Management (Admin)</t>
+          <t>Bulk Kit Auto-Deactivation Cascade Engine</t>
         </is>
       </c>
       <c r="D60" s="13" t="inlineStr">
         <is>
-          <t>boskit-admin/DistributorPlansAdminPage.jsx (81KB)</t>
+          <t>internal-admin-portal/src/portals/admin/pages/solar-shop/warehouse-kit-activations/WarehouseKitConfig.jsx</t>
         </is>
       </c>
       <c r="E60" s="13" t="inlineStr">
         <is>
-          <t>/admin-api/boskit/v1/plans/*</t>
+          <t>/admin-api/solarshop/warehouse-kit-activations/auto-deactivate-bulk, warehouse_kit_activations.handler.js</t>
         </is>
       </c>
       <c r="F60" s="8" t="inlineStr">
@@ -2843,7 +2843,7 @@
       </c>
       <c r="G60" s="14" t="inlineStr">
         <is>
-          <t>Admin management module to configure distributor subscription tiers, security deposits, territory exclusivity rights, and credit policies.</t>
+          <t>Business rule automation engine that cascades deactivations: disabling a Combo Kit in a warehouse automatically disables linked Bulk Kit configurations (autoDeactivateBulkKit) preventing unvalidated wholesale purchases.</t>
         </is>
       </c>
     </row>
@@ -2855,22 +2855,22 @@
       </c>
       <c r="B61" s="5" t="inlineStr">
         <is>
-          <t>BOSKIT</t>
+          <t>Kit Activation &amp; Order Settings</t>
         </is>
       </c>
       <c r="C61" s="6" t="inlineStr">
         <is>
-          <t>Distributor Dashboard</t>
+          <t>District Order Management Scoping (ADM_ORD_MGMT)</t>
         </is>
       </c>
       <c r="D61" s="7" t="inlineStr">
         <is>
-          <t>boskit-website/distributor/DistributorDashboardPage.jsx</t>
+          <t>internal-admin-portal/src/portals/admin/pages/solar-shop/order-management-settings/OrderManagementSettings.jsx</t>
         </is>
       </c>
       <c r="E61" s="7" t="inlineStr">
         <is>
-          <t>GET /api/boskit/v1/distributor/dashboard/stats</t>
+          <t>/admin-api/solarshop/order-settings/*, order_settings.handler.js</t>
         </is>
       </c>
       <c r="F61" s="8" t="inlineStr">
@@ -2880,7 +2880,7 @@
       </c>
       <c r="G61" s="9" t="inlineStr">
         <is>
-          <t>Operational dashboard for BOS distributors to manage local dealer networks, track bulk purchase orders, and monitor regional territory sales.</t>
+          <t>Stage 2 District Fulfillment Configuration supporting Country -&gt; State -&gt; Cluster -&gt; District geographic hierarchy selection with automated Master Warehouse fallback when a district lacks local warehouse facilities.</t>
         </is>
       </c>
     </row>
@@ -2892,22 +2892,22 @@
       </c>
       <c r="B62" s="11" t="inlineStr">
         <is>
-          <t>BOSKIT</t>
+          <t>Kit Activation &amp; Order Settings</t>
         </is>
       </c>
       <c r="C62" s="12" t="inlineStr">
         <is>
-          <t>Distributor Procurement Catalogue</t>
+          <t>Sequential Fulfillment Pipeline Chains</t>
         </is>
       </c>
       <c r="D62" s="13" t="inlineStr">
         <is>
-          <t>boskit-website/distributor/DistributorProcureCataloguePage.jsx</t>
+          <t>internal-admin-portal/src/portals/admin/pages/solar-shop/order-management-settings/OrderManagementSettings.jsx</t>
         </is>
       </c>
       <c r="E62" s="13" t="inlineStr">
         <is>
-          <t>GET /api/boskit/v1/distributor/catalogue</t>
+          <t>/admin-api/solarshop/order-settings/save, order_settings.schema.js</t>
         </is>
       </c>
       <c r="F62" s="8" t="inlineStr">
@@ -2917,7 +2917,7 @@
       </c>
       <c r="G62" s="14" t="inlineStr">
         <is>
-          <t>Wholesale procurement catalog allowing distributors to order BOS components at master trade rates and configure downstream dealer margins.</t>
+          <t>Strict toggle dependency chain enforcement: Combo/Customize Kits (Sub-Warehouse -&gt; Nearest Supplier -&gt; In-Cluster Supplier) and Bulk Kits (Sub-Warehouse -&gt; Master Warehouse -&gt; Nearest Supplier -&gt; In-Cluster Supplier) with automated reverse cascade.</t>
         </is>
       </c>
     </row>
@@ -2929,22 +2929,22 @@
       </c>
       <c r="B63" s="5" t="inlineStr">
         <is>
-          <t>BOSKIT</t>
+          <t>Payments &amp; Accounts</t>
         </is>
       </c>
       <c r="C63" s="6" t="inlineStr">
         <is>
-          <t>Custom BOS Kit Configurator</t>
+          <t>Multi-Order Supplier PO Combination Engine</t>
         </is>
       </c>
       <c r="D63" s="7" t="inlineStr">
         <is>
-          <t>customer-apps/boskit-website/src/pages/BosKitConfigurator.jsx</t>
+          <t>internal-admin-portal/src/portals/accounts/pages/payments/Payments.jsx</t>
         </is>
       </c>
       <c r="E63" s="7" t="inlineStr">
         <is>
-          <t>/api/boskit/v1/configurator</t>
+          <t>/account-api/payments/pending-orders, /account-api/supplier-po/combine, getPendingEpcFranchiseOrders</t>
         </is>
       </c>
       <c r="F63" s="8" t="inlineStr">
@@ -2954,7 +2954,7 @@
       </c>
       <c r="G63" s="9" t="inlineStr">
         <is>
-          <t>Interactive configurator for designing electrical BOS distribution kits tailored to specific inverter capacities and solar string requirements. Interactive BOS kit configurator calculating string sizing, breaker ratings, surge protection, and enclosure specifications.</t>
+          <t>Accounts procurement consolidation engine allowing staff to select multiple pending EPC and Franchise customer orders and combine them into a single consolidated Supplier Purchase Order with auto-calculated BOM cost ratios (Panels ~60%, Inverters ~25%, Others ~15%).</t>
         </is>
       </c>
     </row>
@@ -2966,22 +2966,22 @@
       </c>
       <c r="B64" s="11" t="inlineStr">
         <is>
-          <t>BOSKIT</t>
+          <t>Payments &amp; Accounts</t>
         </is>
       </c>
       <c r="C64" s="12" t="inlineStr">
         <is>
-          <t>Dealer Registration &amp; Dashboard</t>
+          <t>Supplier PO Payment &amp; Tax Invoice Registration</t>
         </is>
       </c>
       <c r="D64" s="13" t="inlineStr">
         <is>
-          <t>boskit-website/dealer/DealerRegisterPage.jsx, DealerDashboardPage.jsx</t>
+          <t>internal-admin-portal/src/portals/accounts/pages/payments/CombinedPaymentModal.jsx</t>
         </is>
       </c>
       <c r="E64" s="13" t="inlineStr">
         <is>
-          <t>/api/boskit/v1/dealer/*</t>
+          <t>/account-api/supplier-po/create-payment, purchase_order.schema.js</t>
         </is>
       </c>
       <c r="F64" s="8" t="inlineStr">
@@ -2991,7 +2991,7 @@
       </c>
       <c r="G64" s="14" t="inlineStr">
         <is>
-          <t>Self-service portal for local electrical dealers to register under regional distributors, browse catalogs, place orders, and track shipments.</t>
+          <t>Comprehensive supplier procurement payment workflow capturing supplier selection, destination warehouse, NEFT/RTGS/UPI reference, payment receipt upload, Proforma Invoice details, and transitional 'paid / awaiting delivery' status tracking.</t>
         </is>
       </c>
     </row>
@@ -3003,22 +3003,22 @@
       </c>
       <c r="B65" s="5" t="inlineStr">
         <is>
-          <t>BOSKIT</t>
+          <t>Warehouse &amp; Logistics</t>
         </is>
       </c>
       <c r="C65" s="6" t="inlineStr">
         <is>
-          <t>BOSKIT Admin Overview &amp; Reports</t>
+          <t>Material Inward &amp; GRN Generation (Inventory Inward)</t>
         </is>
       </c>
       <c r="D65" s="7" t="inlineStr">
         <is>
-          <t>boskit-admin/BoskitOverviewDashboard.jsx, CrossPlatformReportsPage.jsx</t>
+          <t>internal-admin-portal/src/portals/warehouse/pages/material-inward/MaterialInward.jsx (Tab 1)</t>
         </is>
       </c>
       <c r="E65" s="7" t="inlineStr">
         <is>
-          <t>/admin-api/boskit/v1/stats, /reports/*</t>
+          <t>/warehouse-api/material-inward/complete-delivery, inward_log.schema.js</t>
         </is>
       </c>
       <c r="F65" s="8" t="inlineStr">
@@ -3028,7 +3028,7 @@
       </c>
       <c r="G65" s="9" t="inlineStr">
         <is>
-          <t>Executive BI dashboard aggregating channel distribution performance, dealer turnover, and inventory movement across regional BOS networks.</t>
+          <t>Warehouse inward verification workflow recording supplier Tax Invoice No, GSTIN, and PDF upload, auto-generating Goods Receipt Notes (GRN) with QC discrepancy fields (Accepted Qty, Damaged Qty, Shortage notes) and real-time inventory increment.</t>
         </is>
       </c>
     </row>
@@ -3040,32 +3040,32 @@
       </c>
       <c r="B66" s="11" t="inlineStr">
         <is>
-          <t>BOSKIT</t>
+          <t>Warehouse &amp; Logistics</t>
         </is>
       </c>
       <c r="C66" s="12" t="inlineStr">
         <is>
-          <t>BOSKIT MOQ, GST, Channel Settings</t>
+          <t>Customer Order Inward Fulfillment Bridge</t>
         </is>
       </c>
       <c r="D66" s="13" t="inlineStr">
         <is>
-          <t>boskit-admin MoqSettings + GstSettings + ChannelSettings</t>
+          <t>internal-admin-portal/src/portals/warehouse/pages/material-inward/MaterialInward.jsx (Tab 2)</t>
         </is>
       </c>
       <c r="E66" s="13" t="inlineStr">
         <is>
-          <t>/admin-api/boskit/v1/moq-rules/*, tax-rules/*, channel-settings/*</t>
-        </is>
-      </c>
-      <c r="F66" s="8" t="inlineStr">
-        <is>
-          <t>Fully Connected</t>
+          <t>/warehouse-api/order-fulfillment-inward/*, order_inward.handler.js</t>
+        </is>
+      </c>
+      <c r="F66" s="15" t="inlineStr">
+        <is>
+          <t>Partially Connected</t>
         </is>
       </c>
       <c r="G66" s="14" t="inlineStr">
         <is>
-          <t>Platform settings interface managing BOS minimum order quantities, HSN GST tax rules, and channel discount matrices.</t>
+          <t>Supply chain bridge connecting received supplier GRN stock batches to specific pending customer sales orders, validating component availability before releasing orders to the outbound delivery management queue.</t>
         </is>
       </c>
     </row>
@@ -3077,22 +3077,22 @@
       </c>
       <c r="B67" s="5" t="inlineStr">
         <is>
-          <t>BOSKIT</t>
+          <t>Warehouse &amp; Logistics</t>
         </is>
       </c>
       <c r="C67" s="6" t="inlineStr">
         <is>
-          <t>FranchisePlansAdminPage</t>
+          <t>Real-Time FIFO Stock Allocation &amp; Deduction Engine</t>
         </is>
       </c>
       <c r="D67" s="7" t="inlineStr">
         <is>
-          <t>internal-admin-portal/.../boskit/pages/FranchisePlansAdminPage.jsx</t>
+          <t>internal-admin-portal/src/portals/warehouse/pages/delivery-management/DeliveryManagement.jsx</t>
         </is>
       </c>
       <c r="E67" s="7" t="inlineStr">
         <is>
-          <t>Re-exports DistributorPlansAdminPage.jsx (1,604 LOC)</t>
+          <t>/warehouse-api/delivery/fifo-allocate, /warehouse-api/delivery/deduct-stock, warehouse_stock.schema.js</t>
         </is>
       </c>
       <c r="F67" s="8" t="inlineStr">
@@ -3102,7 +3102,7 @@
       </c>
       <c r="G67" s="9" t="inlineStr">
         <is>
-          <t>Dedicated admin interface for managing franchise packages, perks, territory exclusivity clauses, and fee structures (currently a placeholder stub). Comprehensive admin management module for franchise &amp; distributor package pricing, validity, renewal rules, and territory exclusivity.</t>
+          <t>Automated FIFO stock availability inspector evaluating required vs allocated vs shortage quantities for every component in a solar kit BOM, executing atomic inventory deduction upon order delivery completion.</t>
         </is>
       </c>
     </row>
@@ -3563,17 +3563,17 @@
       </c>
       <c r="C80" s="12" t="inlineStr">
         <is>
-          <t>BOSKIT Notifications</t>
+          <t>Delivery &amp; Logistics Milestone Alerts</t>
         </is>
       </c>
       <c r="D80" s="13" t="inlineStr">
         <is>
-          <t>boskit-website notification handler</t>
+          <t>customer-apps/solarkits-reseller-portal, customer-apps/solar-store</t>
         </is>
       </c>
       <c r="E80" s="13" t="inlineStr">
         <is>
-          <t>/api/boskit/v1/notification/*</t>
+          <t>/api/delivery/notifications/*, twilio.service.js, nodemailer.service.js</t>
         </is>
       </c>
       <c r="F80" s="8" t="inlineStr">
@@ -3583,7 +3583,7 @@
       </c>
       <c r="G80" s="14" t="inlineStr">
         <is>
-          <t>Channel communication system alerting distributors and dealers about order dispatches, price revisions, and stock updates.</t>
+          <t>Multi-channel delivery notification engine dispatching automated WhatsApp, SMS, and Email alerts to EPC contractors and Franchisees across key order lifecycle stages (PO Inward, Out for Delivery, Delivered).</t>
         </is>
       </c>
     </row>
@@ -3613,7 +3613,7 @@
           <t>Nodemailer v9 configured in .env</t>
         </is>
       </c>
-      <c r="F81" s="15" t="inlineStr">
+      <c r="F81" s="16" t="inlineStr">
         <is>
           <t>Backend Only</t>
         </is>
@@ -3650,7 +3650,7 @@
           <t>Twilio SDK in package.json</t>
         </is>
       </c>
-      <c r="F82" s="15" t="inlineStr">
+      <c r="F82" s="16" t="inlineStr">
         <is>
           <t>Backend Only</t>
         </is>
@@ -3711,17 +3711,17 @@
       </c>
       <c r="C84" s="12" t="inlineStr">
         <is>
-          <t>BOSKIT Cross-Platform Reports</t>
+          <t>Warehouse Turnaround &amp; Logistics Analytics</t>
         </is>
       </c>
       <c r="D84" s="13" t="inlineStr">
         <is>
-          <t>boskit-admin/CrossPlatformReportsPage.jsx</t>
+          <t>internal-admin-portal/src/portals/warehouse/pages/analytics/WarehouseAnalytics.jsx</t>
         </is>
       </c>
       <c r="E84" s="13" t="inlineStr">
         <is>
-          <t>/admin-api/boskit/v1/reports/*</t>
+          <t>/warehouse-api/analytics/stock-turn, /admin-api/delivery/tat-metrics</t>
         </is>
       </c>
       <c r="F84" s="8" t="inlineStr">
@@ -3731,7 +3731,7 @@
       </c>
       <c r="G84" s="14" t="inlineStr">
         <is>
-          <t>Consolidated reporting engine providing executive visibility across distributor procurement, dealer turnover, and inventory velocity.</t>
+          <t>Executive logistics telemetry evaluating warehouse stock turnover rates, supplier delivery lead times, GRN discrepancy ratios, vehicle cargo load utilization, and average dispatch turnaround time (TAT).</t>
         </is>
       </c>
     </row>
@@ -3798,7 +3798,7 @@
           <t>src/modules/admin-panel/middlewares/mongo.sanitize.js</t>
         </is>
       </c>
-      <c r="F86" s="15" t="inlineStr">
+      <c r="F86" s="16" t="inlineStr">
         <is>
           <t>Backend Only</t>
         </is>
@@ -3835,7 +3835,7 @@
           <t>admin-panel/middlewares/rate.limit.js</t>
         </is>
       </c>
-      <c r="F87" s="15" t="inlineStr">
+      <c r="F87" s="16" t="inlineStr">
         <is>
           <t>Backend Only</t>
         </is>
@@ -3872,7 +3872,7 @@
           <t>cms-auth module, verify_reseller_auth, verify_bde_auth</t>
         </is>
       </c>
-      <c r="F88" s="15" t="inlineStr">
+      <c r="F88" s="16" t="inlineStr">
         <is>
           <t>Backend Only</t>
         </is>
@@ -3909,7 +3909,7 @@
           <t>src/index.js lines 29-45</t>
         </is>
       </c>
-      <c r="F89" s="15" t="inlineStr">
+      <c r="F89" s="16" t="inlineStr">
         <is>
           <t>Backend Only</t>
         </is>
@@ -3946,7 +3946,7 @@
           <t>kycDocUpload middleware in multer</t>
         </is>
       </c>
-      <c r="F90" s="15" t="inlineStr">
+      <c r="F90" s="16" t="inlineStr">
         <is>
           <t>Backend Only</t>
         </is>
@@ -3983,7 +3983,7 @@
           <t>.env.example CLOUDINARY_KYC_UPLOAD_PRESET commented out</t>
         </is>
       </c>
-      <c r="F91" s="15" t="inlineStr">
+      <c r="F91" s="16" t="inlineStr">
         <is>
           <t>Backend Only</t>
         </is>
@@ -4020,7 +4020,7 @@
           <t>Root Dockerfile (5.3KB)</t>
         </is>
       </c>
-      <c r="F92" s="15" t="inlineStr">
+      <c r="F92" s="16" t="inlineStr">
         <is>
           <t>Backend Only</t>
         </is>
@@ -4057,7 +4057,7 @@
           <t>nginx.conf, nginx.prod.conf.template</t>
         </is>
       </c>
-      <c r="F93" s="15" t="inlineStr">
+      <c r="F93" s="16" t="inlineStr">
         <is>
           <t>Backend Only</t>
         </is>
@@ -4415,12 +4415,12 @@
           <t>backend/solarkits-central-backend/src/index.js:45</t>
         </is>
       </c>
-      <c r="E3" s="16" t="inlineStr">
+      <c r="E3" s="17" t="inlineStr">
         <is>
           <t>CRITICAL</t>
         </is>
       </c>
-      <c r="F3" s="17" t="inlineStr">
+      <c r="F3" s="15" t="inlineStr">
         <is>
           <t>Active / In-Progress</t>
         </is>
@@ -4543,39 +4543,39 @@
       </c>
     </row>
     <row r="7">
-      <c r="A7" s="19" t="inlineStr">
+      <c r="A7" s="4" t="inlineStr">
         <is>
           <t>B005</t>
         </is>
       </c>
-      <c r="B7" s="20" t="inlineStr">
-        <is>
-          <t>BOSKIT Admin</t>
-        </is>
-      </c>
-      <c r="C7" s="21" t="inlineStr">
-        <is>
-          <t>FranchisePlansAdminPage.jsx was previously flagged as an empty 111-byte stub</t>
-        </is>
-      </c>
-      <c r="D7" s="22" t="inlineStr">
-        <is>
-          <t>internal-admin-portal/.../boskit/pages/FranchisePlansAdminPage.jsx</t>
-        </is>
-      </c>
-      <c r="E7" s="23" t="inlineStr">
-        <is>
-          <t>MEDIUM</t>
-        </is>
-      </c>
-      <c r="F7" s="24" t="inlineStr">
-        <is>
-          <t>RESOLVED / RETRACTED</t>
-        </is>
-      </c>
-      <c r="G7" s="21" t="inlineStr">
-        <is>
-          <t>AUDIT CLARIFICATION: FranchisePlansAdminPage.jsx is an alias cleanly re-exporting DistributorPlansAdminPage.jsx (1,604 lines of production code) containing full tier, fee, and territory exclusivity controls.</t>
+      <c r="B7" s="5" t="inlineStr">
+        <is>
+          <t>Warehouse Logistics</t>
+        </is>
+      </c>
+      <c r="C7" s="9" t="inlineStr">
+        <is>
+          <t>Material Inward 'Order Inward' tab currently hardcoded with placeholder message and missing backend fulfillment matching</t>
+        </is>
+      </c>
+      <c r="D7" s="7" t="inlineStr">
+        <is>
+          <t>internal-admin-portal/src/portals/warehouse/pages/material-inward/MaterialInward.jsx:activeTab === 'supplier'</t>
+        </is>
+      </c>
+      <c r="E7" s="15" t="inlineStr">
+        <is>
+          <t>HIGH</t>
+        </is>
+      </c>
+      <c r="F7" s="15" t="inlineStr">
+        <is>
+          <t>Active / In-Progress</t>
+        </is>
+      </c>
+      <c r="G7" s="9" t="inlineStr">
+        <is>
+          <t>Tab 1 (Inventory Inward PO delivery &amp; GRN) is fully operational. Tab 2 (Order Inward) is currently under active development to automatically match received GRN stock to source customer sales orders before releasing to delivery.</t>
         </is>
       </c>
     </row>
@@ -4617,39 +4617,39 @@
       </c>
     </row>
     <row r="9">
-      <c r="A9" s="19" t="inlineStr">
+      <c r="A9" s="4" t="inlineStr">
         <is>
           <t>B007</t>
         </is>
       </c>
-      <c r="B9" s="20" t="inlineStr">
-        <is>
-          <t>Solar Store (EPC)</t>
-        </is>
-      </c>
-      <c r="C9" s="21" t="inlineStr">
-        <is>
-          <t>Solar BOS Kit menu item was commented out in navigation</t>
-        </is>
-      </c>
-      <c r="D9" s="22" t="inlineStr">
-        <is>
-          <t>customer-apps/solar-store/src/Pages/dashboard/SolarBosKit.jsx</t>
-        </is>
-      </c>
-      <c r="E9" s="23" t="inlineStr">
-        <is>
-          <t>LOW</t>
-        </is>
-      </c>
-      <c r="F9" s="24" t="inlineStr">
-        <is>
-          <t>RESOLVED</t>
-        </is>
-      </c>
-      <c r="G9" s="21" t="inlineStr">
-        <is>
-          <t>FIXED: SolarBosKit component (1,506 LOC) is fully maintained with dynamic electrical component selection and integrated custom combo kit workflows.</t>
+      <c r="B9" s="5" t="inlineStr">
+        <is>
+          <t>Delivery Logistics</t>
+        </is>
+      </c>
+      <c r="C9" s="9" t="inlineStr">
+        <is>
+          <t>Delivery OTP verification and Proof of Delivery (POD) photo upload UI require mobile/field driver optimization</t>
+        </is>
+      </c>
+      <c r="D9" s="7" t="inlineStr">
+        <is>
+          <t>backend/src/modules/admin-panel/models/india_solarshop_db/delivery_order.schema.js</t>
+        </is>
+      </c>
+      <c r="E9" s="16" t="inlineStr">
+        <is>
+          <t>MEDIUM</t>
+        </is>
+      </c>
+      <c r="F9" s="15" t="inlineStr">
+        <is>
+          <t>Active / In-Progress</t>
+        </is>
+      </c>
+      <c r="G9" s="9" t="inlineStr">
+        <is>
+          <t>Backend fields for OTP confirmation and Cloudinary POD image attachment are implemented in delivery_order.schema.js. Field UI workflows in Operations Tab 8 are undergoing final mobile responsiveness polish.</t>
         </is>
       </c>
     </row>
@@ -4785,12 +4785,12 @@
           <t>internal-admin-portal/.../admin/pages/dashboard/Home.jsx</t>
         </is>
       </c>
-      <c r="E13" s="15" t="inlineStr">
+      <c r="E13" s="16" t="inlineStr">
         <is>
           <t>MEDIUM</t>
         </is>
       </c>
-      <c r="F13" s="17" t="inlineStr">
+      <c r="F13" s="15" t="inlineStr">
         <is>
           <t>Active / In-Progress</t>
         </is>
@@ -4834,7 +4834,7 @@
       </c>
       <c r="G14" s="21" t="inlineStr">
         <is>
-          <t>FIXED: All project documentation updated to formally standardize the Hybrid Dual-Track Architecture: Automated ICICI E-Collection (Virtual Accounts) + Offline Bank Transfer &amp; Payment Receipt Verification.</t>
+          <t>FIXED: All project documentation updated to formally standardize the Hybrid Dual-Track Architecture: Automated ICICI E-Collection (Virtual Accounts) + Offline Bank Transfer &amp; Payment Receipt Verification alongside the 2-Stage Kit Activation &amp; Order Delivery Journey.</t>
         </is>
       </c>
     </row>
@@ -4849,13 +4849,13 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:E7"/>
+  <dimension ref="A1:E9"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="12" customWidth="1" min="1" max="1"/>
-    <col width="18" customWidth="1" min="2" max="2"/>
-    <col width="35" customWidth="1" min="3" max="3"/>
-    <col width="40" customWidth="1" min="4" max="4"/>
+    <col width="20" customWidth="1" min="2" max="2"/>
+    <col width="38" customWidth="1" min="3" max="3"/>
+    <col width="45" customWidth="1" min="4" max="4"/>
     <col width="15" customWidth="1" min="5" max="5"/>
   </cols>
   <sheetData>
@@ -4894,7 +4894,7 @@
       </c>
     </row>
     <row r="3">
-      <c r="A3" s="16" t="inlineStr">
+      <c r="A3" s="17" t="inlineStr">
         <is>
           <t>P0</t>
         </is>
@@ -4911,7 +4911,7 @@
       </c>
       <c r="D3" s="9" t="inlineStr">
         <is>
-          <t>Guarantees strict API access control</t>
+          <t>Guarantees strict API access control &amp; origin validation</t>
         </is>
       </c>
       <c r="E3" s="27" t="inlineStr">
@@ -4938,7 +4938,7 @@
       </c>
       <c r="D4" s="14" t="inlineStr">
         <is>
-          <t>Data privacy compliance for sensitive records</t>
+          <t>Ensures compliance for sensitive customer documents &amp; slips</t>
         </is>
       </c>
       <c r="E4" s="30" t="inlineStr">
@@ -4948,81 +4948,135 @@
       </c>
     </row>
     <row r="5">
-      <c r="A5" s="17" t="inlineStr">
+      <c r="A5" s="15" t="inlineStr">
         <is>
           <t>P1</t>
         </is>
       </c>
       <c r="B5" s="5" t="inlineStr">
         <is>
-          <t>Admin Panel</t>
+          <t>Warehouse Logistics</t>
         </is>
       </c>
       <c r="C5" s="26" t="inlineStr">
         <is>
-          <t>Complete central Admin Dashboard Home.jsx executive overview metrics</t>
+          <t>Build 'Order Inward' tab backend matching logic linking received GRN stock to customer orders</t>
         </is>
       </c>
       <c r="D5" s="9" t="inlineStr">
         <is>
-          <t>Real-time network KPIs for Super Admin</t>
+          <t>Completes the critical bridge between supplier procurement &amp; customer dispatch</t>
         </is>
       </c>
       <c r="E5" s="27" t="inlineStr">
         <is>
+          <t>High</t>
+        </is>
+      </c>
+    </row>
+    <row r="6">
+      <c r="A6" s="18" t="inlineStr">
+        <is>
+          <t>P1</t>
+        </is>
+      </c>
+      <c r="B6" s="11" t="inlineStr">
+        <is>
+          <t>Delivery Logistics</t>
+        </is>
+      </c>
+      <c r="C6" s="29" t="inlineStr">
+        <is>
+          <t>Complete mobile Delivery OTP verification and Proof of Delivery (POD) photo upload UI</t>
+        </is>
+      </c>
+      <c r="D6" s="14" t="inlineStr">
+        <is>
+          <t>Provides tamper-proof delivery verification for drivers and warehouse staff</t>
+        </is>
+      </c>
+      <c r="E6" s="30" t="inlineStr">
+        <is>
           <t>Medium</t>
-        </is>
-      </c>
-    </row>
-    <row r="6">
-      <c r="A6" s="31" t="inlineStr">
-        <is>
-          <t>P2</t>
-        </is>
-      </c>
-      <c r="B6" s="11" t="inlineStr">
-        <is>
-          <t>Documentation</t>
-        </is>
-      </c>
-      <c r="C6" s="29" t="inlineStr">
-        <is>
-          <t>Publish Swagger / OpenAPI 3.0 API specifications for all 10 modules</t>
-        </is>
-      </c>
-      <c r="D6" s="14" t="inlineStr">
-        <is>
-          <t>Accelerates developer onboarding &amp; QA audits</t>
-        </is>
-      </c>
-      <c r="E6" s="30" t="inlineStr">
-        <is>
-          <t>Large</t>
         </is>
       </c>
     </row>
     <row r="7">
       <c r="A7" s="15" t="inlineStr">
         <is>
+          <t>P1</t>
+        </is>
+      </c>
+      <c r="B7" s="5" t="inlineStr">
+        <is>
+          <t>Admin Panel</t>
+        </is>
+      </c>
+      <c r="C7" s="26" t="inlineStr">
+        <is>
+          <t>Complete central Admin Dashboard Home.jsx executive overview metrics</t>
+        </is>
+      </c>
+      <c r="D7" s="9" t="inlineStr">
+        <is>
+          <t>Delivers real-time network KPIs, revenue, and active orders for Super Admin</t>
+        </is>
+      </c>
+      <c r="E7" s="27" t="inlineStr">
+        <is>
+          <t>Medium</t>
+        </is>
+      </c>
+    </row>
+    <row r="8">
+      <c r="A8" s="31" t="inlineStr">
+        <is>
           <t>P2</t>
         </is>
       </c>
-      <c r="B7" s="5" t="inlineStr">
-        <is>
-          <t>Testing</t>
-        </is>
-      </c>
-      <c r="C7" s="26" t="inlineStr">
-        <is>
-          <t>Establish automated integration test suite with Jest / Supertest</t>
-        </is>
-      </c>
-      <c r="D7" s="9" t="inlineStr">
-        <is>
-          <t>Continuous regression protection for payments</t>
-        </is>
-      </c>
-      <c r="E7" s="27" t="inlineStr">
+      <c r="B8" s="11" t="inlineStr">
+        <is>
+          <t>Supplier Portal</t>
+        </is>
+      </c>
+      <c r="C8" s="29" t="inlineStr">
+        <is>
+          <t>Implement supplier self-service Proforma Invoice submission &amp; PO confirmation workflow</t>
+        </is>
+      </c>
+      <c r="D8" s="14" t="inlineStr">
+        <is>
+          <t>Accelerates supplier procurement lifecycle and removes manual coordination</t>
+        </is>
+      </c>
+      <c r="E8" s="30" t="inlineStr">
+        <is>
+          <t>Medium</t>
+        </is>
+      </c>
+    </row>
+    <row r="9">
+      <c r="A9" s="16" t="inlineStr">
+        <is>
+          <t>P2</t>
+        </is>
+      </c>
+      <c r="B9" s="5" t="inlineStr">
+        <is>
+          <t>Testing &amp; QA</t>
+        </is>
+      </c>
+      <c r="C9" s="26" t="inlineStr">
+        <is>
+          <t>Establish automated integration test suite with Jest / Supertest for ICICI SSE, PO combinations &amp; FIFO stock deduction</t>
+        </is>
+      </c>
+      <c r="D9" s="9" t="inlineStr">
+        <is>
+          <t>Continuous regression protection for critical commercial &amp; logistics pipelines</t>
+        </is>
+      </c>
+      <c r="E9" s="27" t="inlineStr">
         <is>
           <t>Large</t>
         </is>
@@ -5042,12 +5096,12 @@
   <dimension ref="A1:F15"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
-    <col width="28" customWidth="1" min="1" max="1"/>
+    <col width="32" customWidth="1" min="1" max="1"/>
     <col width="12" customWidth="1" min="2" max="2"/>
     <col width="12" customWidth="1" min="3" max="3"/>
     <col width="12" customWidth="1" min="4" max="4"/>
     <col width="20" customWidth="1" min="5" max="5"/>
-    <col width="50" customWidth="1" min="6" max="6"/>
+    <col width="55" customWidth="1" min="6" max="6"/>
   </cols>
   <sheetData>
     <row r="1" ht="25" customHeight="1">
@@ -5070,7 +5124,7 @@
       </c>
       <c r="C2" s="2" t="inlineStr">
         <is>
-          <t>Sep 25 %</t>
+          <t>Oct 10 %</t>
         </is>
       </c>
       <c r="D2" s="2" t="inlineStr">
@@ -5092,7 +5146,7 @@
     <row r="3">
       <c r="A3" s="32" t="inlineStr">
         <is>
-          <t>Backend API (all 10 modules)</t>
+          <t>Backend API (all 10 domain modules)</t>
         </is>
       </c>
       <c r="B3" s="33" t="inlineStr">
@@ -5284,32 +5338,32 @@
     <row r="9">
       <c r="A9" s="32" t="inlineStr">
         <is>
-          <t>BOSKIT B2B Platform</t>
+          <t>Kit Activation &amp; Order Settings</t>
         </is>
       </c>
       <c r="B9" s="33" t="inlineStr">
         <is>
-          <t>68%</t>
+          <t>75%</t>
         </is>
       </c>
       <c r="C9" s="34" t="inlineStr">
         <is>
-          <t>80%</t>
+          <t>92%</t>
         </is>
       </c>
       <c r="D9" s="35" t="inlineStr">
         <is>
-          <t>+12.0%</t>
+          <t>+17.0%</t>
         </is>
       </c>
       <c r="E9" s="32" t="inlineStr">
         <is>
-          <t>Substantial Progress</t>
+          <t>Production Ready</t>
         </is>
       </c>
       <c r="F9" s="36" t="inlineStr">
         <is>
-          <t>Franchise plans re-export verified (1,604 LOC), distributor catalog, dealer ordering</t>
+          <t>2-stage pipeline: Warehouse 3-gate validation + District sequential fulfillment routing (Sub-WH -&gt; Nearest -&gt; In-Cluster)</t>
         </is>
       </c>
     </row>
@@ -5341,7 +5395,7 @@
       </c>
       <c r="F10" s="41" t="inlineStr">
         <is>
-          <t>Dual-track engine: ICICI Automated E-Collection + Offline Bank Transfer &amp; Verification</t>
+          <t>Multi-Order Supplier PO combination modal, ICICI Automated E-Collection + Offline Bank Transfer &amp; Verification</t>
         </is>
       </c>
     </row>
@@ -5373,14 +5427,14 @@
       </c>
       <c r="F11" s="36" t="inlineStr">
         <is>
-          <t>Inward logging, stock reservation, fleet drivers/vehicles, repair ticket schema</t>
+          <t>Material Inward GRN logging, supplier PO delivery, FIFO BOM allocation, fleet drivers/vehicles, repair ticket schema</t>
         </is>
       </c>
     </row>
     <row r="12">
       <c r="A12" s="37" t="inlineStr">
         <is>
-          <t>Operations Module</t>
+          <t>Operations &amp; Delivery Module</t>
         </is>
       </c>
       <c r="B12" s="38" t="inlineStr">
@@ -5390,12 +5444,12 @@
       </c>
       <c r="C12" s="39" t="inlineStr">
         <is>
-          <t>80%</t>
+          <t>82%</t>
         </is>
       </c>
       <c r="D12" s="40" t="inlineStr">
         <is>
-          <t>+50.0%</t>
+          <t>+52.0%</t>
         </is>
       </c>
       <c r="E12" s="37" t="inlineStr">
@@ -5405,14 +5459,14 @@
       </c>
       <c r="F12" s="41" t="inlineStr">
         <is>
-          <t>Delivery Queue Tab 7, Trip Tracking Tab 8, automated vehicle recommendation engine</t>
+          <t>8-Stage delivery pipeline, Delivery Queue Tab 7, Trip POD Tab 8, automated vehicle recommendation engine</t>
         </is>
       </c>
     </row>
     <row r="13">
       <c r="A13" s="32" t="inlineStr">
         <is>
-          <t>Reports &amp; Analytics</t>
+          <t>Reports &amp; Logistics Analytics</t>
         </is>
       </c>
       <c r="B13" s="33" t="inlineStr">
@@ -5437,7 +5491,7 @@
       </c>
       <c r="F13" s="36" t="inlineStr">
         <is>
-          <t>BDE conversion funnel, monthly target tracking, delivery TAT and cargo metrics</t>
+          <t>BDE conversion funnel, monthly target tracking, delivery TAT and warehouse turnaround metrics</t>
         </is>
       </c>
     </row>
@@ -5501,7 +5555,7 @@
       </c>
       <c r="F15" s="47" t="inlineStr">
         <is>
-          <t>Production-ready stage; major commercial supply chain &amp; banking integrations complete</t>
+          <t>Production-ready stage; major commercial supply chain, 2-stage kit activation &amp; banking integrations complete</t>
         </is>
       </c>
     </row>

</xml_diff>